<commit_message>
708pm update - 092826
</commit_message>
<xml_diff>
--- a/source/Current Pricelist - HPNB.xlsx
+++ b/source/Current Pricelist - HPNB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhonedcel_nolasco\Desktop\Test Pilot - HP Pricelist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78489E58-22B2-4CEB-A027-8D2DC520D501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB45EF43-BE68-4B20-B6D6-910DB3B03F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{46EB8EAC-1B53-4337-BC93-2BB462C6E864}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="66">
   <si>
     <t>HP 15</t>
   </si>
@@ -208,9 +208,6 @@
     <t>SRP</t>
   </si>
   <si>
-    <t>Qty</t>
-  </si>
-  <si>
     <t>DP</t>
   </si>
   <si>
@@ -233,6 +230,12 @@
   </si>
   <si>
     <t>Promo DP</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Onhand</t>
   </si>
 </sst>
 </file>
@@ -279,9 +282,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -13173,10 +13175,10 @@
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
         <v>51</v>
@@ -13194,13 +13196,13 @@
         <v>55</v>
       </c>
       <c r="I2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K2" t="s">
         <v>64</v>
-      </c>
-      <c r="K2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
@@ -13208,7 +13210,7 @@
         <f>_xlfn.XLOOKUP(F3,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DM8L5PA</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <f>VLOOKUP(B3,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036894</v>
       </c>
@@ -13224,16 +13226,16 @@
       <c r="G3" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>56990</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <f>H3*0.85</f>
         <v>48441.5</v>
       </c>
-      <c r="J3" s="2"/>
-      <c r="K3">
-        <v>69</v>
+      <c r="J3" s="1"/>
+      <c r="K3" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
@@ -13241,7 +13243,7 @@
         <f>_xlfn.XLOOKUP(F4,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DJ8T8PA</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <f>VLOOKUP(B4,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036895</v>
       </c>
@@ -13257,16 +13259,16 @@
       <c r="G4" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>62990</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <f t="shared" ref="I4:I23" si="0">H4*0.85</f>
         <v>53541.5</v>
       </c>
-      <c r="J4" s="2"/>
-      <c r="K4">
-        <v>705</v>
+      <c r="J4" s="1"/>
+      <c r="K4" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
@@ -13274,7 +13276,7 @@
         <f>_xlfn.XLOOKUP(F5,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5U6PA</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <f>VLOOKUP(B5,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036897</v>
       </c>
@@ -13290,16 +13292,16 @@
       <c r="G5" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>58990</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <f t="shared" si="0"/>
         <v>50141.5</v>
       </c>
-      <c r="J5" s="2"/>
-      <c r="K5">
-        <v>150</v>
+      <c r="J5" s="1"/>
+      <c r="K5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
@@ -13307,7 +13309,7 @@
         <f>_xlfn.XLOOKUP(F6,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DW4U8PA</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <f>VLOOKUP(B6,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036898</v>
       </c>
@@ -13315,7 +13317,7 @@
         <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -13323,19 +13325,19 @@
       <c r="G6" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>60990</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <f t="shared" si="0"/>
         <v>51841.5</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <f t="shared" ref="J6:J11" si="1">H6*0.8</f>
         <v>48792</v>
       </c>
-      <c r="K6">
-        <v>250</v>
+      <c r="K6" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -13343,7 +13345,7 @@
         <f>_xlfn.XLOOKUP(F7,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DW4U9PA</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <f>VLOOKUP(B7,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036899</v>
       </c>
@@ -13351,7 +13353,7 @@
         <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
         <v>9</v>
@@ -13359,19 +13361,19 @@
       <c r="G7" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>60990</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <f t="shared" si="0"/>
         <v>51841.5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <f t="shared" si="1"/>
         <v>48792</v>
       </c>
-      <c r="K7">
-        <v>250</v>
+      <c r="K7" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -13379,7 +13381,7 @@
         <f>_xlfn.XLOOKUP(F8,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DW7W9PA</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <f>VLOOKUP(B8,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036900</v>
       </c>
@@ -13387,7 +13389,7 @@
         <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
         <v>11</v>
@@ -13395,19 +13397,19 @@
       <c r="G8" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>64990</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <f t="shared" si="0"/>
         <v>55241.5</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <f t="shared" si="1"/>
         <v>51992</v>
       </c>
-      <c r="K8">
-        <v>875</v>
+      <c r="K8" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
@@ -13415,7 +13417,7 @@
         <f>_xlfn.XLOOKUP(F9,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DJ8T4PA</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <f>VLOOKUP(B9,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036903</v>
       </c>
@@ -13423,7 +13425,7 @@
         <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
         <v>13</v>
@@ -13431,19 +13433,19 @@
       <c r="G9" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>85990</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <f t="shared" si="0"/>
         <v>73091.5</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <f t="shared" si="1"/>
         <v>68792</v>
       </c>
-      <c r="K9">
-        <v>290</v>
+      <c r="K9" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
@@ -13451,7 +13453,7 @@
         <f>_xlfn.XLOOKUP(F10,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DX4J7PA</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <f>VLOOKUP(B10,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036904</v>
       </c>
@@ -13459,7 +13461,7 @@
         <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F10" t="s">
         <v>15</v>
@@ -13467,19 +13469,19 @@
       <c r="G10" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>87990</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <f t="shared" si="0"/>
         <v>74791.5</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <f t="shared" si="1"/>
         <v>70392</v>
       </c>
-      <c r="K10">
-        <v>196</v>
+      <c r="K10" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
@@ -13487,7 +13489,7 @@
         <f>_xlfn.XLOOKUP(F11,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5R6PA</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <f>VLOOKUP(B11,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036907</v>
       </c>
@@ -13495,7 +13497,7 @@
         <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F11" t="s">
         <v>17</v>
@@ -13503,19 +13505,19 @@
       <c r="G11" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>80990</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <f t="shared" si="0"/>
         <v>68841.5</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <f t="shared" si="1"/>
         <v>64792</v>
       </c>
-      <c r="K11">
-        <v>170</v>
+      <c r="K11" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
@@ -13523,7 +13525,7 @@
         <f>_xlfn.XLOOKUP(F12,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5S6PA</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <f>VLOOKUP(B12,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036914</v>
       </c>
@@ -13531,7 +13533,7 @@
         <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F12" t="s">
         <v>19</v>
@@ -13539,16 +13541,16 @@
       <c r="G12" t="s">
         <v>20</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>103990</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <f t="shared" si="0"/>
         <v>88391.5</v>
       </c>
-      <c r="J12" s="2"/>
-      <c r="K12">
-        <v>152</v>
+      <c r="J12" s="1"/>
+      <c r="K12" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -13556,7 +13558,7 @@
         <f>_xlfn.XLOOKUP(F13,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5S7PA</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="2">
         <f>VLOOKUP(B13,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036915</v>
       </c>
@@ -13564,7 +13566,7 @@
         <v>49</v>
       </c>
       <c r="E13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" t="s">
         <v>21</v>
@@ -13572,16 +13574,16 @@
       <c r="G13" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>113990</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <f t="shared" si="0"/>
         <v>96891.5</v>
       </c>
-      <c r="J13" s="2"/>
-      <c r="K13">
-        <v>50</v>
+      <c r="J13" s="1"/>
+      <c r="K13" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -13589,7 +13591,7 @@
         <f>_xlfn.XLOOKUP(F14,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5T2PA</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <f>VLOOKUP(B14,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036916</v>
       </c>
@@ -13597,7 +13599,7 @@
         <v>49</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F14" t="s">
         <v>23</v>
@@ -13605,16 +13607,16 @@
       <c r="G14" t="s">
         <v>24</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>138990</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <f t="shared" si="0"/>
         <v>118141.5</v>
       </c>
-      <c r="J14" s="2"/>
-      <c r="K14">
-        <v>10</v>
+      <c r="J14" s="1"/>
+      <c r="K14" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -13622,7 +13624,7 @@
         <f>_xlfn.XLOOKUP(F15,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5S8PA</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="2">
         <f>VLOOKUP(B15,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036917</v>
       </c>
@@ -13630,7 +13632,7 @@
         <v>49</v>
       </c>
       <c r="E15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F15" t="s">
         <v>25</v>
@@ -13638,16 +13640,16 @@
       <c r="G15" t="s">
         <v>26</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>159990</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <f t="shared" si="0"/>
         <v>135991.5</v>
       </c>
-      <c r="J15" s="2"/>
-      <c r="K15">
-        <v>9</v>
+      <c r="J15" s="1"/>
+      <c r="K15" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
@@ -13655,7 +13657,7 @@
         <f>_xlfn.XLOOKUP(F16,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5T6PA</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="2">
         <f>VLOOKUP(B16,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036919</v>
       </c>
@@ -13663,7 +13665,7 @@
         <v>50</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F16" t="s">
         <v>27</v>
@@ -13671,16 +13673,16 @@
       <c r="G16" t="s">
         <v>28</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>101990</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <f t="shared" si="0"/>
         <v>86691.5</v>
       </c>
-      <c r="J16" s="2"/>
-      <c r="K16">
-        <v>15</v>
+      <c r="J16" s="1"/>
+      <c r="K16" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
@@ -13688,7 +13690,7 @@
         <f>_xlfn.XLOOKUP(F17,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5S1PA</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="2">
         <f>VLOOKUP(B17,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036922</v>
       </c>
@@ -13696,7 +13698,7 @@
         <v>49</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F17" t="s">
         <v>29</v>
@@ -13704,16 +13706,16 @@
       <c r="G17" t="s">
         <v>30</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>112990</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <f t="shared" si="0"/>
         <v>96041.5</v>
       </c>
-      <c r="J17" s="2"/>
-      <c r="K17">
-        <v>236</v>
+      <c r="J17" s="1"/>
+      <c r="K17" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
@@ -13721,7 +13723,7 @@
         <f>_xlfn.XLOOKUP(F18,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5S4PA</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="2">
         <f>VLOOKUP(B18,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036923</v>
       </c>
@@ -13729,7 +13731,7 @@
         <v>49</v>
       </c>
       <c r="E18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F18" t="s">
         <v>31</v>
@@ -13737,16 +13739,16 @@
       <c r="G18" t="s">
         <v>32</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>122990</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="1">
         <f t="shared" si="0"/>
         <v>104541.5</v>
       </c>
-      <c r="J18" s="2"/>
-      <c r="K18">
-        <v>95</v>
+      <c r="J18" s="1"/>
+      <c r="K18" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
@@ -13754,7 +13756,7 @@
         <f>_xlfn.XLOOKUP(F19,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5S5PA</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="2">
         <f>VLOOKUP(B19,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036924</v>
       </c>
@@ -13762,7 +13764,7 @@
         <v>49</v>
       </c>
       <c r="E19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F19" t="s">
         <v>33</v>
@@ -13770,16 +13772,16 @@
       <c r="G19" t="s">
         <v>34</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>169990</v>
       </c>
-      <c r="I19" s="2">
+      <c r="I19" s="1">
         <f t="shared" si="0"/>
         <v>144491.5</v>
       </c>
-      <c r="J19" s="2"/>
-      <c r="K19">
-        <v>5</v>
+      <c r="J19" s="1"/>
+      <c r="K19" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.25">
@@ -13787,7 +13789,7 @@
         <f>_xlfn.XLOOKUP(F20,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5T4PA</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="2">
         <f>VLOOKUP(B20,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036925</v>
       </c>
@@ -13795,7 +13797,7 @@
         <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F20" t="s">
         <v>35</v>
@@ -13803,16 +13805,16 @@
       <c r="G20" t="s">
         <v>36</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>106990</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I20" s="1">
         <f t="shared" si="0"/>
         <v>90941.5</v>
       </c>
-      <c r="J20" s="2"/>
-      <c r="K20">
-        <v>249</v>
+      <c r="J20" s="1"/>
+      <c r="K20" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.25">
@@ -13820,7 +13822,7 @@
         <f>_xlfn.XLOOKUP(F21,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DW8J8PA</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="2">
         <f>VLOOKUP(B21,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036926</v>
       </c>
@@ -13828,7 +13830,7 @@
         <v>50</v>
       </c>
       <c r="E21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F21" t="s">
         <v>37</v>
@@ -13836,16 +13838,16 @@
       <c r="G21" t="s">
         <v>38</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>109990</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21" s="1">
         <f t="shared" si="0"/>
         <v>93491.5</v>
       </c>
-      <c r="J21" s="2"/>
-      <c r="K21">
-        <v>50</v>
+      <c r="J21" s="1"/>
+      <c r="K21" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.25">
@@ -13853,7 +13855,7 @@
         <f>_xlfn.XLOOKUP(F22,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DU5T3PA</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="2">
         <f>VLOOKUP(B22,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036927</v>
       </c>
@@ -13861,7 +13863,7 @@
         <v>50</v>
       </c>
       <c r="E22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F22" t="s">
         <v>39</v>
@@ -13869,16 +13871,16 @@
       <c r="G22" t="s">
         <v>40</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>158990</v>
       </c>
-      <c r="I22" s="2">
+      <c r="I22" s="1">
         <f t="shared" si="0"/>
         <v>135141.5</v>
       </c>
-      <c r="J22" s="2"/>
-      <c r="K22">
-        <v>10</v>
+      <c r="J22" s="1"/>
+      <c r="K22" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
@@ -13886,7 +13888,7 @@
         <f>_xlfn.XLOOKUP(F23,'[1]non-gaming'!$G:$G,'[1]non-gaming'!$D:$D)</f>
         <v>DM8L6PA</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23" s="2">
         <f>VLOOKUP(B23,'[2]ZMATINFO NB - 0924'!$N:$R,4,0)</f>
         <v>432115036971</v>
       </c>
@@ -13902,16 +13904,16 @@
       <c r="G23" t="s">
         <v>42</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>57990</v>
       </c>
-      <c r="I23" s="2">
+      <c r="I23" s="1">
         <f t="shared" si="0"/>
         <v>49291.5</v>
       </c>
-      <c r="J23" s="2"/>
-      <c r="K23" s="1">
-        <v>2267</v>
+      <c r="J23" s="1"/>
+      <c r="K23" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>